<commit_message>
feat: enhance analyst review process with validation status and writeback functionality
- Updated comparison schema version to 3 to accommodate new features.
- Added new fields for validation status, reviewer, and review date in Excel output.
- Implemented a function to extract and format analyst review fields from comparison items.
- Enhanced row collection logic to include analyst review data for various change types.
- Introduced a new module for persisting analyst decisions back to comparison.json and regenerating comparison.xlsx.
- Ensured that previous review decisions are stripped before applying new ones to maintain data integrity.
- Added logging for writeback operations to track success and failures.
</commit_message>
<xml_diff>
--- a/outputs/resultats/bmo/2025_t2_vs_2025_t1/comparison.xlsx
+++ b/outputs/resultats/bmo/2025_t2_vs_2025_t1/comparison.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changements détectés" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changements détectés'!$A$1:$K$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changements détectés'!$A$1:$N$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -471,6 +471,9 @@
     <col width="70" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -529,26 +532,41 @@
           <t>Commentaire analyste</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Statut validation</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Validé par</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Validé le</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gestion du capital</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>TABLEAU 13</t>
+          <t>(sans titre)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>44</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -563,17 +581,19 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le nombre d’actions ordinaires est présenté déduction faite de 95 889 actions propres.</t>
+          <t>À la suite des hausses des taux d’intérêt, le portefeuille comprenait des prêts hypothécaires à taux variables à amortissement négatif totalisant 2,6 milliards de dollars (9,3 milliards au 31 octobre 2024) les paiements contractuels de la période considérée étant appliqués aux intérêts et la portion des intérêts exigibles non visée par des versements étant appliquée au capital.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Convertible en actions ordinaires. Les billets avec remboursement de capital à recours limité sont convertibles en actions ordinaires en vertu du recours aux actions privilégiées, série 49, aux actions privilégiées, série 51, aux actions privilégiées, série 53 et aux actions privilégiées, série 54 au titre des billets avec remboursement de capital à recours limité, série 3, série 4 et série 5, respectivement émises en même temps que les billets avec remboursement de capital à recours limité, qui comprennent actuellement une clause de non-viabilité limitée.</t>
+          <t>À la suite des hausses des taux d’intérêt, le portefeuille comprenait des prêts hypothécaires à taux variables à amortissement négatif totalisant 0,1 milliard de dollars (2,6 milliards au 31 janvier 2025) les paiements contractuels de la période considérée étant appliqués aux intérêts et la portion des intérêts exigibles non visée par des versements étant appliquée au capital.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>This change significantly alters the understanding of the financial instruments' characteristics, impacting regulatory compliance and investor information.</t>
+          <t>La note de bas de page n°3 a été modifiée dans le tableau de répartition de la période d’amortissement des prêts hypothécaires. Le texte a été révisé pour indiquer que le montant total des prêts hypothécaires à taux variables à amortissement négatif est passé de 2,6 milliards de dollars à 0,1 milliard de dollars. Cette modification est significative car elle reflète une réduction substantielle du portefeuille de prêts à amortissement négatif.
+Ce changement a un impact direct sur l'évaluation du risque de crédit et la gestion des actifs de la banque. Une diminution aussi drastique du montant des prêts à amortissement négatif pourrait indiquer une amélioration de la qualité du portefeuille ou une modification des pratiques de gestion des risques. Selon les normes de Bâle III, une telle réduction pourrait influencer les exigences de fonds propres en réduisant le risque pondéré des actifs.
+Il s'agit d'une divulgation critique qui nécessite une attention particulière. L'analyste devrait confirmer la raison de cette réduction et s'assurer que les pratiques de gestion des risques sont alignées avec les politiques internes et les exigences réglementaires. Une investigation plus approfondie est recommandée pour comprendre les implications de cette modification sur la stratégie de gestion des risques de la banque.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -582,59 +602,79 @@
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-18T19:07:11.697494+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>(sans titre)</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>TABLEAU 13</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Note de bas de page</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Modification</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>À la suite des hausses des taux d’intérêt, le portefeuille comprenait des prêts hypothécaires à taux variables à amortissement négatif totalisant 2,6 milliards de dollars (9,3 milliards au 31 octobre 2024) les paiements contractuels de la période considérée étant appliqués aux intérêts et la portion des intérêts exigibles non visée par des versements étant appliquée au capital.</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>À la suite des hausses des taux d’intérêt, le portefeuille comprenait des prêts hypothécaires à taux variables à amortissement négatif totalisant 0,1 milliard de dollars (2,6 milliards au 31 janvier 2025) les paiements contractuels de la période considérée étant appliqués aux intérêts et la portion des intérêts exigibles non visée par des versements étant appliquée au capital.</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>The substantial decrease in the reported amount of negative amortization mortgages from 2.6 billion to 0.1 billion indicates a significant change in the bank's risk exposure and financial position, necessitating further analysis.</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Le nombre d’actions ordinaires est présenté déduction faite de 95 889 actions propres.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Convertible en actions ordinaires. Les billets avec remboursement de capital à recours limité sont convertibles en actions ordinaires en vertu du recours aux actions privilégiées, série 49, aux actions privilégiées, série 51, aux actions privilégiées, série 53 et aux actions privilégiées, série 54 au titre des billets avec remboursement de capital à recours limité, série 3, série 4 et série 5, respectivement émises en même temps que les billets avec remboursement de capital à recours limité, qui comprennent actuellement une clause de non-viabilité limitée.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>La note de bas de page n°2 a subi une révision matérielle dans le tableau des actions en circulation et titres convertibles en actions ordinaires au T2 2025.
+Initialement, cette note indiquait simplement le nombre d'actions ordinaires déduction faite des actions propres. La nouvelle version de la note fournit des détails complexes sur la convertibilité des billets avec remboursement de capital à recours limité en actions ordinaires, en précisant les séries d'actions privilégiées concernées et l'inclusion d'une clause de non-viabilité limitée. Ce changement a des implications significatives pour la compréhension des mécanismes de conversion et des conditions associées, ce qui est crucial pour l'évaluation des risques et la conformité réglementaire.
+Il s'agit d'une divulgation critique et potentiellement réglementaire. L'analyste devrait escalader cette révision pour s'assurer que toutes les implications réglementaires et de risque sont correctement évaluées et que la divulgation est conforme aux exigences de transparence du BSIF et de Bâle III.</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -679,7 +719,9 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The removal of 'prêts automobiles et de prêts au financement de matériel de transport' from the scope of securitizations indicates a significant change in the asset composition, which could impact risk assessments and financial reporting.</t>
+          <t>La note de bas de page n-3 a été modifiée dans le tableau des échéances du financement de gros. Le texte précédent mentionnait que les titrisations comprenaient les créances de cartes de crédit, de prêts automobiles et de prêts au financement de matériel de transport. Dans la version actuelle, seules les créances de cartes de crédit sont mentionnées.
+Ce changement réduit le périmètre des actifs titrisés pris en compte dans le calcul du financement de gros. Cela peut avoir un impact sur les ratios de liquidité et de capital, notamment en ce qui concerne les exigences de Bâle III sur la titrisation et la gestion des risques de crédit. La réduction des types de créances titrisées pourrait indiquer un changement dans la stratégie de financement ou une réévaluation des risques associés à certains types d'actifs.
+Il s'agit d'un changement méthodologique significatif qui pourrait affecter la perception du risque de crédit et de liquidité de l'institution. L'analyste devrait investiguer les raisons de cette modification et s'assurer que les ajustements sont cohérents avec les autres divulgations financières et les politiques de gestion des risques de l'institution.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -688,6 +730,21 @@
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18T19:06:53.369119+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -697,38 +754,44 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>TABLEAU 38</t>
+          <t>TABLEAU 36</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>47</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>51</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Indicateur</t>
+          <t>Note de bas de page</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Suppression</t>
+          <t>Modification</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Instruments financiers inscrits au bilan</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr"/>
+          <t>2 Les valeurs sont calculées en fonction de la moyenne simple du RLCT quotidien sur 62 jours ouvrables au premier trimestre de 2025.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>2 Les valeurs sont calculées en fonction de la moyenne simple du RLCT quotidien sur 61 jours ouvrables au deuxième trimestre de l’exercice 2025.</t>
+        </is>
+      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The removal of the 'Instruments financiers inscrits au bilan' indicator suggests a structural change in how financial instruments are reported, potentially impacting the clarity of financial disclosures.</t>
+          <t>La note de bas de page numéro 2 a subi une modification dans le tableau du ratio de liquidité à court terme. Le texte a été ajusté pour indiquer que les valeurs sont désormais calculées sur une moyenne simple du RLCT quotidien sur 61 jours ouvrables au deuxième trimestre de l’exercice 2025, au lieu de 62 jours au premier trimestre de 2025.
+Ce changement a un impact direct sur la méthodologie de calcul du ratio de liquidité à court terme, un indicateur clé de la gestion des risques de liquidité. La réduction du nombre de jours ouvrables pris en compte peut affecter la précision et la comparabilité des ratios entre les trimestres. Cela pourrait également avoir des implications sur la conformité avec les exigences réglementaires, notamment celles du BSIF, qui stipulent des normes précises pour le calcul des ratios de liquidité.
+Il s'agit d'un changement méthodologique significatif. L'analyste devrait investiguer la raison de cette modification et s'assurer que la nouvelle méthodologie est cohérente avec les autres pratiques de calcul de la liquidité de la banque. Une vérification de la conformité avec les directives du BSIF est également recommandée.</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -737,6 +800,21 @@
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18T19:07:17.439778+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -746,17 +824,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>TABLEAU 41</t>
+          <t>TABLEAU 38</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>49</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>53</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -777,7 +855,9 @@
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The removal of the 'Instruments financiers inscrits au bilan' indicator suggests a structural change in how financial instruments are reported, potentially impacting the clarity of financial disclosures.</t>
+          <t>L'indicateur "Instruments financiers inscrits au bilan" a été supprimé du tableau des échéances des actifs d’instruments financiers inscrits au bilan au T2 2025, alors qu'il était présent au T1 2025.
+Cette suppression peut indiquer un changement dans la manière dont les actifs financiers sont présentés ou catégorisés dans le rapport. L'indicateur servait probablement de titre ou de catégorie englobante pour les actifs financiers inscrits au bilan, et sa disparition pourrait refléter une simplification ou une réorganisation de la présentation des données. Cela pourrait avoir un impact sur la compréhension des lecteurs quant à la structure des actifs financiers de l'institution.
+Il s'agit d'un changement structurel dans la présentation des données. L'analyste devrait vérifier si cette suppression est compensée par une autre forme de présentation ou si elle résulte d'une modification méthodologique. Il est recommandé de confirmer que les informations essentielles sont toujours couvertes ailleurs dans le rapport.</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -786,26 +866,41 @@
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr"/>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18T19:07:36.604467+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Gestion du capital</t>
+          <t>Gestion des risques</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>TABLEAU 13</t>
+          <t>TABLEAU 41</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>50</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>54</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -815,18 +910,20 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Ajout</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Série N – première tranche</t>
-        </is>
-      </c>
+          <t>Suppression</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Instruments financiers inscrits au bilan</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The addition of a new series of securities ('Série N – première tranche') could indicate a structural change in the capital management strategy, potentially affecting the bank's capital structure and investor relations.</t>
+          <t>L'indicateur "Instruments financiers inscrits au bilan" a été retiré du tableau des échéances des instruments financiers inscrits au bilan au T2 2025, alors qu'il était présent au T1 2025.
+Ce retrait peut indiquer un changement dans la présentation des informations financières, potentiellement lié à une réorganisation des catégories d'actifs ou à une mise à jour des normes de divulgation. Bien que cet indicateur ne soit pas directement lié à une exigence réglementaire spécifique comme Bâle III, il joue un rôle dans la transparence des informations fournies aux parties prenantes.
+Il s'agit probablement d'une mise à jour structurelle du tableau. L'analyste devrait vérifier si cette information est désormais intégrée ailleurs dans le rapport ou si elle a été jugée redondante.</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -835,6 +932,21 @@
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18T19:07:02.577910+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -859,27 +971,25 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Note de bas de page</t>
+          <t>Indicateur</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Convertible en actions ordinaires. Les billets avec remboursement de capital à recours limité sont convertibles en actions ordinaires en vertu du recours aux actions privilégiées, série 49, aux actions privilégiées, série 51, aux actions privilégiées, série 53 et aux actions privilégiées, série 54 au titre des billets avec remboursement de capital à recours limité, série 3, série 4 et série 5, respectivement émises en même temps que les billets avec remboursement de capital à recours limité, qui comprennent actions privilégiées à recours limité.</t>
-        </is>
-      </c>
+          <t>Ajout</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Les billets avaient un taux d’intérêt initial de 4,800 %, qui a été ajusté à 6,709 % le 25 août 2024.</t>
+          <t>Série N – première tranche</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>This change affects the understanding of financial terms and conditions, which is important for financial analysis and investor decision-making.</t>
+          <t>L'indicateur "Série N – première tranche" a été ajouté dans le tableau de gestion du capital au T2 2025, alors qu'il était absent au T1 2025.
+Cet ajout pourrait indiquer l'émission de nouveaux titres ou une nouvelle catégorisation des instruments financiers. Cela peut avoir un impact sur la structure du capital de la banque, influençant potentiellement les ratios de fonds propres réglementaires tels que ceux définis par Bâle III. La divulgation de ces informations est cruciale pour assurer la transparence vis-à-vis des investisseurs et des régulateurs.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer la nature de cette nouvelle série et s'assurer que les valeurs associées sont correctement intégrées dans les calculs des ratios de fonds propres.</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -888,6 +998,21 @@
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18T19:06:38.303790+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -917,18 +1042,24 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Suppression</t>
+          <t>Modification</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
+          <t>Convertible en actions ordinaires. Les billets avec remboursement de capital à recours limité sont convertibles en actions ordinaires en vertu du recours aux actions privilégiées, série 49, aux actions privilégiées, série 51, aux actions privilégiées, série 53 et aux actions privilégiées, série 54 au titre des billets avec remboursement de capital à recours limité, série 3, série 4 et série 5, respectivement émises en même temps que les billets avec remboursement de capital à recours limité, qui comprennent actions privilégiées à recours limité.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
           <t>Les billets avaient un taux d’intérêt initial de 4,800 %, qui a été ajusté à 6,709 % le 25 août 2024.</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The removal of this footnote could impact the understanding of interest rate adjustments on specific financial instruments, which is crucial for accurate financial analysis and reporting.</t>
+          <t>La note de bas de page n°3 a été révisée de manière significative dans le tableau des actions en circulation et titres convertibles en actions ordinaires au T2 2025.
+La version précédente de cette note décrivait la convertibilité des billets avec remboursement de capital à recours limité en actions ordinaires, en détaillant les séries d'actions privilégiées impliquées. La nouvelle version se concentre sur l'ajustement du taux d'intérêt des billets, passant de 4,800 % à 6,709 % à une date précise. Ce changement de focus modifie la nature de l'information divulguée, passant d'une explication sur la structure de capital à une mise à jour sur les conditions financières des instruments de dette.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que cette révision est correctement reflétée dans les autres sections du rapport et que les implications sur les coûts de financement et les ratios de fonds propres sont bien comprises et communiquées.</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -937,55 +1068,63 @@
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr"/>
+      <c r="M9" s="3" t="inlineStr"/>
+      <c r="N9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>TABLEAU 36</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>51</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Indicateur</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>TABLEAU 13</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Note de bas de page</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Suppression</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Pour le trimestre clos le 31 octobre 2024 – Total des sorties nettes de trésorerie</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>The removal of this indicator may reflect a change in reporting format, but it is likely cosmetic as the core data is still represented.</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Les billets avaient un taux d’intérêt initial de 4,800 %, qui a été ajusté à 6,709 % le 25 août 2024.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>La note de bas de page n°4 a été supprimée du tableau des actions en circulation et titres convertibles en actions ordinaires au T2 2025.
+Cette note précisait un ajustement du taux d'intérêt des billets subordonnés, passant de 4,800 % à 6,709 % à une date spécifique. La suppression de cette information pourrait avoir des implications sur la transparence des conditions financières des instruments de dette de la banque, ce qui est crucial pour les investisseurs et les régulateurs. Les ajustements de taux d'intérêt peuvent affecter les coûts de financement et, par conséquent, les ratios de fonds propres réglementaires tels que définis par Bâle III.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer si cette information est désormais incluse ailleurs dans le rapport ou si elle a été omise par erreur. Une vérification de la cohérence des divulgations sur les taux d'intérêt est recommandée.</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr"/>
+      <c r="N10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -995,38 +1134,44 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>TABLEAU 36</t>
+          <t>(sans titre)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>44</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>48</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Indicateur</t>
+          <t>Note de bas de page</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Suppression</t>
+          <t>Modification</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Pour le trimestre clos le 31 octobre 2024 – Ratio de liquidité à court terme (%)</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr"/>
+          <t>Les autres actifs non grevés comprennent certains actifs liquides qui, de l’avis de la direction, ne sont pas rapidement disponibles pour répondre aux besoins de BMO en matière de liquidité. Ces actifs se composent de valeurs mobilières d’un montant de 25,9 milliards de dollars au 31 janvier 2025 et comprennent les titres détenus par la filiale d’assurance de BMO, les titres liés au financement par le vendeur et certains investissements détenus par notre unité de banque d’affaires. Les autres actifs non grevés comprennent des prêts hypothécaires et d’autres prêts pouvant être titrisés afin d’obtenir du financement garanti.</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Les autres actifs non grevés comprennent certains actifs liquides qui, de l’avis de la direction, ne sont pas rapidement disponibles pour répondre aux besoins de BMO en matière de liquidité. Ces actifs se composent de valeurs mobilières d’un montant de 24,9 milliards de dollars au 30 avril 2025 et comprennent les titres détenus par la filiale d’assurance de BMO, les titres liés au financement par le vendeur et certains investissements détenus par notre unité de banque d’affaires. Les autres actifs non grevés comprennent des prêts hypothécaires et d’autres prêts pouvant être titrisés afin d’obtenir du financement garanti.</t>
+        </is>
+      </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>The removal of this indicator may reflect a change in reporting format, but it is likely cosmetic as the core data is still represented.</t>
+          <t>La note de bas de page n°3 a subi une modification mineure dans le tableau des actifs grevés et non grevés. Le changement concerne uniquement la mise à jour du montant des valeurs mobilières, passant de 25,9 milliards de dollars au 31 janvier 2025 à 24,9 milliards de dollars au 30 avril 2025. Cette modification est purement quantitative et ne modifie pas la nature ou la portée des actifs décrits.
+D'un point de vue réglementaire et métier, cette mise à jour n'a pas d'impact significatif. Elle reflète simplement une variation normale des valeurs mobilières détenues par la banque, ce qui est courant dans la gestion des actifs et des liquidités. Il n'y a pas de nouvelles exigences de divulgation ou de changement de méthodologie impliqués ici, et cela ne touche pas aux ratios prudentiels ou aux exigences de Bâle III.
+En conclusion, ce changement est une mise à jour ordinaire des chiffres financiers sans implication méthodologique ou réglementaire. L'analyste peut confirmer cette mise à jour sans nécessiter d'investigation supplémentaire ou d'escalade. Il est recommandé de vérifier la cohérence de ces chiffres avec d'autres sections du rapport pour assurer l'exactitude globale des données financières.</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1035,54 +1180,328 @@
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr"/>
+      <c r="M11" s="4" t="inlineStr"/>
+      <c r="N11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>TABLEAU 34</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Note de bas de page</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Le total du financement de gros était constitué de 52,3 milliards de dollars de fonds libellés en dollars canadiens et de 211,1 milliards de fonds libellés en dollars américains et en d’autres monnaies au 31 janvier 2025.</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Le total du financement de gros était constitué de 53,0 milliards de dollars de fonds libellés en dollars canadiens et de 205,8 milliards de fonds libellés en dollars américains et en d’autres monnaies au 30 avril 2025.</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>La note de bas de page n-4 a été mise à jour pour refléter les nouvelles valeurs du financement de gros en dollars canadiens et en devises étrangères. Les montants sont passés de 52,3 milliards à 53,0 milliards de dollars canadiens et de 211,1 milliards à 205,8 milliards de dollars américains et autres monnaies.
+Ce changement est principalement une mise à jour des chiffres financiers pour le trimestre en cours. Il reflète les variations dans la composition monétaire du financement de gros, ce qui peut être dû à des fluctuations de change ou à des ajustements dans la stratégie de financement de l'institution. Bien que ces chiffres soient importants pour l'analyse financière, ils ne représentent pas un changement méthodologique ou réglementaire.
+Il s'agit d'une mise à jour ordinaire des données financières. L'analyste devrait confirmer que ces chiffres sont cohérents avec les autres sections du rapport financier et qu'ils reflètent fidèlement la situation financière actuelle de l'institution.</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr"/>
+      <c r="N12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>TABLEAU 39</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Note de bas de page</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Des dépôts de 29 063 millions de dollars au 31 janvier 2025 ont une date d’échéance fixe, mais ils peuvent toutefois faire l’objet d’une demande de remboursement anticipé (en totalité ou en partie) par le client sans pénalité. Ils sont classés comme étant exigibles à une date fixe en raison de leur date d’échéance contractuelle déclarée.</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Des dépôts de 28 685 millions de dollars au 30 avril 2025 ont une date d’échéance fixe, mais ils peuvent toutefois faire l’objet d’une demande de remboursement anticipé (en totalité ou en partie) par le client sans pénalité. Ils sont classés comme étant exigibles à une date fixe en raison de leur date d’échéance contractuelle déclarée.</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>La note de bas de page n°3 a été mise à jour pour refléter un changement de montant et de date, passant de 29 063 millions de dollars au 31 janvier 2025 à 28 685 millions de dollars au 30 avril 2025. Cette note est liée aux dépôts ayant une date d’échéance fixe mais pouvant être remboursés anticipativement.
+Ce changement est purement factuel et reflète une mise à jour des données financières pour le trimestre en cours. Il n'affecte pas la méthodologie de calcul des échéances ni les obligations de divulgation réglementaire. Les principes de classification restent inchangés, conformément aux normes IFRS et aux directives du BSIF.
+Il s'agit d'une mise à jour ordinaire des données financières. L'analyste peut confirmer que cette modification est conforme aux pratiques de mise à jour trimestrielle et ne nécessite pas d'investigation supplémentaire.</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr"/>
+      <c r="M13" s="4" t="inlineStr"/>
+      <c r="N13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>TABLEAU 42</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Note de bas de page</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Les prêts à vue sont inclus dans la colonne Sans échéance.</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Les prêts à vue sont inclus dans la colonne Sans échéance spécifique.</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>La note de bas de page n°1 a subi une légère modification de formulation, passant de 'Sans échéance' à 'Sans échéance spécifique'. Cette modification concerne le tableau des échéances des passifs et capitaux propres, qui est un élément clé de la gestion des risques de liquidité de la banque.
+Bien que le changement de formulation semble mineur, il pourrait refléter une tentative de clarification de la terminologie utilisée pour décrire les échéances des prêts à vue. Cela pourrait avoir un impact sur la manière dont les informations sont interprétées par les parties prenantes, mais il n'y a pas d'implication réglementaire directe ou de changement méthodologique apparent lié à Bâle III ou aux exigences du BSIF.
+Ce changement est principalement cosmétique et vise à améliorer la clarté du rapport. L'analyste devrait confirmer que cette modification n'entraîne pas de confusion supplémentaire et qu'elle est cohérente avec d'autres sections du rapport.</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr"/>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-18T19:06:51.386666+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>TABLEAU 42</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Note de bas de page</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Les dépôts à vue et à préavis sont inclus dans la colonne Sans échéance.</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Les dépôts à vue et à préavis sont inclus dans la colonne Sans échéance spécifique.</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>La note de bas de page n°2 a été modifiée pour inclure le terme 'spécifique' après 'Sans échéance'. Cette modification apparaît dans le même tableau des échéances des passifs et capitaux propres, qui est essentiel pour l'analyse de la liquidité et des engagements de la banque.
+L'ajout du mot 'spécifique' semble être une clarification terminologique sans impact direct sur les calculs ou les ratios prudentiels. Il n'y a pas de changement dans la méthodologie de calcul des échéances ou des dépôts, et cela ne semble pas affecter les exigences de divulgation réglementaire.
+Ce changement est considéré comme cosmétique et vise à améliorer la précision du langage utilisé dans le rapport. L'analyste devrait s'assurer que cette modification est bien comprise par les lecteurs du rapport et qu'elle est appliquée de manière cohérente dans d'autres documents connexes.</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-18T19:07:34.344781+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
           <t>Réglementation</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>TABLEAU 21</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Tableau</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Suppression</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>TABLEAU 21</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Tableau supprimé du trimestre courant.</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-18T19:07:26.977810+00:00</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K12"/>
+  <autoFilter ref="A1:N16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor footnote comparison logic for improved matching accuracy
- Updated the footnote diff calculation to match by normalized text rather than ID, allowing for better handling of renumbered footnotes.
- Enhanced the logic to identify modified footnotes when the same ID is retained but the text changes.
- Removed redundant code related to cross-matching removed and added footnotes by text similarity.
- Adjusted the generated timestamp in the manifest file to reflect the latest update.
- Updated the comparison results in the Excel output file.
</commit_message>
<xml_diff>
--- a/outputs/resultats/bmo/2025_t2_vs_2025_t1/comparison.xlsx
+++ b/outputs/resultats/bmo/2025_t2_vs_2025_t1/comparison.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changements détectés" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changements détectés'!$A$1:$N$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changements détectés'!$A$1:$N$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -591,9 +591,9 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>La note de bas de page n°3 a été modifiée dans le tableau de répartition de la période d’amortissement des prêts hypothécaires. Le texte a été révisé pour indiquer que le montant total des prêts hypothécaires à taux variables à amortissement négatif est passé de 2,6 milliards de dollars à 0,1 milliard de dollars. Cette modification est significative car elle reflète une réduction substantielle du portefeuille de prêts à amortissement négatif.
-Ce changement a un impact direct sur l'évaluation du risque de crédit et la gestion des actifs de la banque. Une diminution aussi drastique du montant des prêts à amortissement négatif pourrait indiquer une amélioration de la qualité du portefeuille ou une modification des pratiques de gestion des risques. Selon les normes de Bâle III, une telle réduction pourrait influencer les exigences de fonds propres en réduisant le risque pondéré des actifs.
-Il s'agit d'une divulgation critique qui nécessite une attention particulière. L'analyste devrait confirmer la raison de cette réduction et s'assurer que les pratiques de gestion des risques sont alignées avec les politiques internes et les exigences réglementaires. Une investigation plus approfondie est recommandée pour comprendre les implications de cette modification sur la stratégie de gestion des risques de la banque.</t>
+          <t>La note de bas de page n°3 a subi une modification significative dans le tableau de répartition de la période d’amortissement des prêts hypothécaires. Le montant total des prêts hypothécaires à taux variables à amortissement négatif est passé de 2,6 milliards de dollars à 0,1 milliard de dollars, ce qui représente une réduction drastique de l'exposition à ce type de produit financier risqué.
+Cette modification a un impact direct sur l'évaluation du risque de crédit et la gestion des risques de la banque. Les prêts à amortissement négatif sont souvent considérés comme plus risqués, car ils peuvent entraîner une augmentation du solde du prêt si les paiements ne couvrent pas les intérêts dus. Une réduction aussi importante pourrait indiquer une amélioration de la qualité du portefeuille ou une modification de la stratégie de gestion des risques. Selon les normes de Bâle III, une telle réduction pourrait également influencer les exigences de fonds propres réglementaires, car elle affecte le profil de risque global de la banque.
+Il s'agit d'une divulgation critique qui nécessite une attention particulière. L'analyste devrait confirmer la raison de cette réduction et s'assurer que les ajustements sont correctement reflétés dans les autres sections du rapport financier. Une enquête plus approfondie pourrait être nécessaire pour comprendre les implications de cette réduction sur la stratégie de gestion des risques de la banque.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -614,67 +614,63 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-18T19:07:11.697494+00:00</t>
+          <t>2026-04-19T00:10:59.190392+00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>TABLEAU 13</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>TABLEAU 27</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Note de bas de page</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Le nombre d’actions ordinaires est présenté déduction faite de 95 889 actions propres.</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Convertible en actions ordinaires. Les billets avec remboursement de capital à recours limité sont convertibles en actions ordinaires en vertu du recours aux actions privilégiées, série 49, aux actions privilégiées, série 51, aux actions privilégiées, série 53 et aux actions privilégiées, série 54 au titre des billets avec remboursement de capital à recours limité, série 3, série 4 et série 5, respectivement émises en même temps que les billets avec remboursement de capital à recours limité, qui comprennent actuellement une clause de non-viabilité limitée.</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>La note de bas de page n°2 a subi une révision matérielle dans le tableau des actions en circulation et titres convertibles en actions ordinaires au T2 2025.
-Initialement, cette note indiquait simplement le nombre d'actions ordinaires déduction faite des actions propres. La nouvelle version de la note fournit des détails complexes sur la convertibilité des billets avec remboursement de capital à recours limité en actions ordinaires, en précisant les séries d'actions privilégiées concernées et l'inclusion d'une clause de non-viabilité limitée. Ce changement a des implications significatives pour la compréhension des mécanismes de conversion et des conditions associées, ce qui est crucial pour l'évaluation des risques et la conformité réglementaire.
-Il s'agit d'une divulgation critique et potentiellement réglementaire. L'analyste devrait escalader cette révision pour s'assurer que toutes les implications réglementaires et de risque sont correctement évaluées et que la divulgation est conforme aux exigences de transparence du BSIF et de Bâle III.</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Ajout</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Certains chiffres comparatifs ont été reclassés en fonction de la présentation adoptée pour la période à l’étude.</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>La note de bas de page n-3 a été ajoutée dans le tableau des liens entre éléments du bilan et risque de marché au T2 2025.
+Cette note précise que certains chiffres comparatifs ont été reclassés selon la nouvelle présentation adoptée pour la période à l’étude. Cela indique un changement dans la manière dont les données sont présentées, ce qui peut avoir un impact sur l'analyse des tendances et la comparabilité des données d'une période à l'autre.
+Il s'agit d'un changement structurel important. L'analyste devrait confirmer que ce reclassement est conforme aux normes comptables applicables et vérifier si d'autres tableaux du rapport ont subi des modifications similaires. Une attention particulière doit être portée à l'impact potentiel sur les ratios financiers et les indicateurs de performance clés.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr"/>
+      <c r="M3" s="3" t="inlineStr"/>
+      <c r="N3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -720,8 +716,8 @@
       <c r="I4" s="3" t="inlineStr">
         <is>
           <t>La note de bas de page n-3 a été modifiée dans le tableau des échéances du financement de gros. Le texte précédent mentionnait que les titrisations comprenaient les créances de cartes de crédit, de prêts automobiles et de prêts au financement de matériel de transport. Dans la version actuelle, seules les créances de cartes de crédit sont mentionnées.
-Ce changement réduit le périmètre des actifs titrisés pris en compte dans le calcul du financement de gros. Cela peut avoir un impact sur les ratios de liquidité et de capital, notamment en ce qui concerne les exigences de Bâle III sur la titrisation et la gestion des risques de crédit. La réduction des types de créances titrisées pourrait indiquer un changement dans la stratégie de financement ou une réévaluation des risques associés à certains types d'actifs.
-Il s'agit d'un changement méthodologique significatif qui pourrait affecter la perception du risque de crédit et de liquidité de l'institution. L'analyste devrait investiguer les raisons de cette modification et s'assurer que les ajustements sont cohérents avec les autres divulgations financières et les politiques de gestion des risques de l'institution.</t>
+Ce changement réduit le périmètre des actifs titrisés inclus dans le calcul, ce qui peut avoir un impact sur la perception du risque associé à ces actifs. En termes de gestion des risques et de conformité réglementaire, cela pourrait affecter les ratios de capital et les exigences de divulgation selon les normes de Bâle III, notamment en ce qui concerne la pondération des actifs par le risque.
+Il s'agit d'un changement structurel important qui pourrait indiquer une révision de la stratégie de titrisation de la banque. L'analyste devrait confirmer la raison de cette modification et s'assurer qu'elle est cohérente avec les autres divulgations financières et les stratégies de gestion des risques de la banque.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -742,7 +738,7 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>2026-04-18T19:06:53.369119+00:00</t>
+          <t>2026-04-19T00:10:36.694576+00:00</t>
         </is>
       </c>
     </row>
@@ -789,9 +785,9 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>La note de bas de page numéro 2 a subi une modification dans le tableau du ratio de liquidité à court terme. Le texte a été ajusté pour indiquer que les valeurs sont désormais calculées sur une moyenne simple du RLCT quotidien sur 61 jours ouvrables au deuxième trimestre de l’exercice 2025, au lieu de 62 jours au premier trimestre de 2025.
-Ce changement a un impact direct sur la méthodologie de calcul du ratio de liquidité à court terme, un indicateur clé de la gestion des risques de liquidité. La réduction du nombre de jours ouvrables pris en compte peut affecter la précision et la comparabilité des ratios entre les trimestres. Cela pourrait également avoir des implications sur la conformité avec les exigences réglementaires, notamment celles du BSIF, qui stipulent des normes précises pour le calcul des ratios de liquidité.
-Il s'agit d'un changement méthodologique significatif. L'analyste devrait investiguer la raison de cette modification et s'assurer que la nouvelle méthodologie est cohérente avec les autres pratiques de calcul de la liquidité de la banque. Une vérification de la conformité avec les directives du BSIF est également recommandée.</t>
+          <t>La note de bas de page numéro 2 a été modifiée dans le tableau du ratio de liquidité à court terme. Le texte précédent indiquait que les valeurs étaient calculées sur une moyenne simple du RLCT quotidien sur 62 jours ouvrables au premier trimestre de 2025. Le texte actuel précise que cette moyenne est désormais calculée sur 61 jours ouvrables au deuxième trimestre de l’exercice 2025.
+Ce changement a un impact direct sur la méthodologie de calcul du ratio de liquidité à court terme, un indicateur clé de la gestion des risques de liquidité. La modification du nombre de jours ouvrables pris en compte peut affecter la précision et la comparabilité des ratios de liquidité, ce qui est crucial pour les exigences de divulgation réglementaire sous Bâle III et les lignes directrices du BSIF.
+Il s'agit d'un changement méthodologique significatif. L'analyste devrait investiguer la raison de cette modification dans le calcul et s'assurer que cette nouvelle méthodologie est cohérente avec les autres sections du rapport et conforme aux exigences réglementaires.</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -800,21 +796,9 @@
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr"/>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-18T19:07:17.439778+00:00</t>
-        </is>
-      </c>
+      <c r="L5" s="3" t="inlineStr"/>
+      <c r="M5" s="3" t="inlineStr"/>
+      <c r="N5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -856,8 +840,8 @@
       <c r="I6" s="3" t="inlineStr">
         <is>
           <t>L'indicateur "Instruments financiers inscrits au bilan" a été supprimé du tableau des échéances des actifs d’instruments financiers inscrits au bilan au T2 2025, alors qu'il était présent au T1 2025.
-Cette suppression peut indiquer un changement dans la manière dont les actifs financiers sont présentés ou catégorisés dans le rapport. L'indicateur servait probablement de titre ou de catégorie englobante pour les actifs financiers inscrits au bilan, et sa disparition pourrait refléter une simplification ou une réorganisation de la présentation des données. Cela pourrait avoir un impact sur la compréhension des lecteurs quant à la structure des actifs financiers de l'institution.
-Il s'agit d'un changement structurel dans la présentation des données. L'analyste devrait vérifier si cette suppression est compensée par une autre forme de présentation ou si elle résulte d'une modification méthodologique. Il est recommandé de confirmer que les informations essentielles sont toujours couvertes ailleurs dans le rapport.</t>
+Cette suppression peut indiquer un changement dans la manière dont les actifs financiers sont présentés ou catégorisés dans le rapport. L'indicateur servait probablement de titre ou de catégorie englobante pour les actifs financiers inscrits au bilan, et son absence pourrait refléter une simplification ou une réorganisation de la présentation des données.
+Il s'agit d'un changement structurel qui pourrait affecter la compréhension globale du tableau par les parties prenantes. L'analyste devrait confirmer que cette suppression n'entraîne pas de perte d'information critique et que les autres indicateurs du tableau couvrent adéquatement les informations précédemment englobées par cet indicateur.</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -878,7 +862,7 @@
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>2026-04-18T19:07:36.604467+00:00</t>
+          <t>2026-04-19T00:10:46.154438+00:00</t>
         </is>
       </c>
     </row>
@@ -921,9 +905,9 @@
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>L'indicateur "Instruments financiers inscrits au bilan" a été retiré du tableau des échéances des instruments financiers inscrits au bilan au T2 2025, alors qu'il était présent au T1 2025.
-Ce retrait peut indiquer un changement dans la présentation des informations financières, potentiellement lié à une réorganisation des catégories d'actifs ou à une mise à jour des normes de divulgation. Bien que cet indicateur ne soit pas directement lié à une exigence réglementaire spécifique comme Bâle III, il joue un rôle dans la transparence des informations fournies aux parties prenantes.
-Il s'agit probablement d'une mise à jour structurelle du tableau. L'analyste devrait vérifier si cette information est désormais intégrée ailleurs dans le rapport ou si elle a été jugée redondante.</t>
+          <t>L'indicateur "Instruments financiers inscrits au bilan" a été supprimé du tableau actuel des échéances contractuelles des actifs, alors qu'il était présent dans le tableau précédent des échéances des instruments financiers inscrits au bilan.
+Cette suppression peut indiquer un changement dans la manière dont les actifs sont présentés ou catégorisés dans le rapport. L'indicateur supprimé servait probablement de titre ou de catégorie englobante pour les actifs inscrits au bilan, ce qui pourrait avoir des implications sur la clarté et la structure de la présentation des données financières.
+Il s'agit d'un changement structurel qui pourrait affecter la compréhension des données par les parties prenantes. L'analyste devrait vérifier si cette suppression est compensée par une autre forme de présentation ou si elle nécessite une clarification supplémentaire dans le rapport.</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -932,21 +916,9 @@
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr"/>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-18T19:07:02.577910+00:00</t>
-        </is>
-      </c>
+      <c r="L7" s="3" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr"/>
+      <c r="N7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -987,9 +959,9 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>L'indicateur "Série N – première tranche" a été ajouté dans le tableau de gestion du capital au T2 2025, alors qu'il était absent au T1 2025.
-Cet ajout pourrait indiquer l'émission de nouveaux titres ou une nouvelle catégorisation des instruments financiers. Cela peut avoir un impact sur la structure du capital de la banque, influençant potentiellement les ratios de fonds propres réglementaires tels que ceux définis par Bâle III. La divulgation de ces informations est cruciale pour assurer la transparence vis-à-vis des investisseurs et des régulateurs.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer la nature de cette nouvelle série et s'assurer que les valeurs associées sont correctement intégrées dans les calculs des ratios de fonds propres.</t>
+          <t>L'indicateur 'Série N – première tranche' a été ajouté dans le tableau de gestion du capital au T2 2025, alors qu'il était absent au T1 2025.
+Cet ajout pourrait indiquer l'émission d'une nouvelle série de titres ou d'instruments financiers, ce qui peut avoir un impact sur la structure du capital de la banque. Cela pourrait également refléter une stratégie de financement ou de gestion des risques modifiée, en lien avec les exigences de fonds propres réglementaires telles que définies par Bâle III ou les lignes directrices du BSIF.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer la nature de cet ajout et s'assurer qu'il est correctement intégré dans les calculs de fonds propres et de ratios prudentiels.</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -1010,7 +982,7 @@
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>2026-04-18T19:06:38.303790+00:00</t>
+          <t>2026-04-19T00:10:15.112415+00:00</t>
         </is>
       </c>
     </row>
@@ -1047,19 +1019,19 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Convertible en actions ordinaires. Les billets avec remboursement de capital à recours limité sont convertibles en actions ordinaires en vertu du recours aux actions privilégiées, série 49, aux actions privilégiées, série 51, aux actions privilégiées, série 53 et aux actions privilégiées, série 54 au titre des billets avec remboursement de capital à recours limité, série 3, série 4 et série 5, respectivement émises en même temps que les billets avec remboursement de capital à recours limité, qui comprennent actions privilégiées à recours limité.</t>
+          <t>Le nombre d’actions ordinaires est présenté déduction faite de 95 889 actions propres.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Les billets avaient un taux d’intérêt initial de 4,800 %, qui a été ajusté à 6,709 % le 25 août 2024.</t>
+          <t>Convertible en actions ordinaires. Les billets avec remboursement de capital à recours limité sont convertibles en actions ordinaires en vertu du recours aux actions privilégiées, série 49, aux actions privilégiées, série 51, aux actions privilégiées, série 53 et aux actions privilégiées, série 54 au titre des billets avec remboursement de capital à recours limité, série 3, série 4 et série 5, respectivement émises en même temps que les billets avec remboursement de capital à recours limité, qui comprennent actuellement une clause de non-viabilité limitée.</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>La note de bas de page n°3 a été révisée de manière significative dans le tableau des actions en circulation et titres convertibles en actions ordinaires au T2 2025.
-La version précédente de cette note décrivait la convertibilité des billets avec remboursement de capital à recours limité en actions ordinaires, en détaillant les séries d'actions privilégiées impliquées. La nouvelle version se concentre sur l'ajustement du taux d'intérêt des billets, passant de 4,800 % à 6,709 % à une date précise. Ce changement de focus modifie la nature de l'information divulguée, passant d'une explication sur la structure de capital à une mise à jour sur les conditions financières des instruments de dette.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que cette révision est correctement reflétée dans les autres sections du rapport et que les implications sur les coûts de financement et les ratios de fonds propres sont bien comprises et communiquées.</t>
+          <t>La note de bas de page n°2 a subi une révision matérielle dans le tableau des actions en circulation et des titres convertibles en actions ordinaires au T2 2025. Le texte précédent mentionnait simplement le nombre d'actions ordinaires déduction faite des actions propres, tandis que le texte révisé détaille les conditions de conversion des billets avec remboursement de capital à recours limité en actions ordinaires.
+Cette révision est significative car elle introduit des informations cruciales sur les mécanismes de conversion et les clauses de non-viabilité, qui sont essentielles pour l'évaluation des risques de capital et la conformité aux exigences de Bâle III. Les investisseurs et les régulateurs s'appuient sur ces informations pour comprendre les implications des instruments financiers sur la structure du capital de la banque.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que cette révision est cohérente avec les autres divulgations du rapport et s'assurer que toutes les implications réglementaires sont correctement adressées.</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -1068,9 +1040,21 @@
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr"/>
-      <c r="L9" s="3" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr"/>
-      <c r="N9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-19T00:11:18.100025+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1105,15 +1089,15 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Les billets avaient un taux d’intérêt initial de 4,800 %, qui a été ajusté à 6,709 % le 25 août 2024.</t>
+          <t>Convertible en actions ordinaires. Les billets avec remboursement de capital à recours limité sont convertibles en actions ordinaires en vertu du recours aux actions privilégiées, série 49, aux actions privilégiées, série 51, aux actions privilégiées, série 53 et aux actions privilégiées, série 54 au titre des billets avec remboursement de capital à recours limité, série 3, série 4 et série 5, respectivement émises en même temps que les billets avec remboursement de capital à recours limité, qui comprennent actions privilégiées à recours limité.</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr"/>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>La note de bas de page n°4 a été supprimée du tableau des actions en circulation et titres convertibles en actions ordinaires au T2 2025.
-Cette note précisait un ajustement du taux d'intérêt des billets subordonnés, passant de 4,800 % à 6,709 % à une date spécifique. La suppression de cette information pourrait avoir des implications sur la transparence des conditions financières des instruments de dette de la banque, ce qui est crucial pour les investisseurs et les régulateurs. Les ajustements de taux d'intérêt peuvent affecter les coûts de financement et, par conséquent, les ratios de fonds propres réglementaires tels que définis par Bâle III.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer si cette information est désormais incluse ailleurs dans le rapport ou si elle a été omise par erreur. Une vérification de la cohérence des divulgations sur les taux d'intérêt est recommandée.</t>
+          <t>La note de bas de page n°3 a été supprimée du tableau des actions en circulation et des titres convertibles en actions ordinaires au T2 2025. Cette note expliquait les conditions de conversion des billets avec remboursement de capital à recours limité en actions ordinaires, en précisant les séries d'actions privilégiées concernées.
+La suppression de cette note pourrait avoir un impact sur la transparence des informations fournies aux investisseurs et aux régulateurs concernant les mécanismes de conversion des instruments financiers. Cela pourrait également affecter la compréhension des conditions de non-viabilité associées à ces instruments, qui sont cruciales pour l'évaluation des risques de capital selon les normes de Bâle III et les directives du BSIF.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer si cette suppression est compensée par une divulgation ailleurs dans le rapport ou si elle nécessite une clarification supplémentaire pour maintenir la conformité réglementaire.</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
@@ -1122,9 +1106,21 @@
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr"/>
-      <c r="L10" s="3" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr"/>
-      <c r="N10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-19T00:11:43.591641+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1169,9 +1165,9 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>La note de bas de page n°3 a subi une modification mineure dans le tableau des actifs grevés et non grevés. Le changement concerne uniquement la mise à jour du montant des valeurs mobilières, passant de 25,9 milliards de dollars au 31 janvier 2025 à 24,9 milliards de dollars au 30 avril 2025. Cette modification est purement quantitative et ne modifie pas la nature ou la portée des actifs décrits.
-D'un point de vue réglementaire et métier, cette mise à jour n'a pas d'impact significatif. Elle reflète simplement une variation normale des valeurs mobilières détenues par la banque, ce qui est courant dans la gestion des actifs et des liquidités. Il n'y a pas de nouvelles exigences de divulgation ou de changement de méthodologie impliqués ici, et cela ne touche pas aux ratios prudentiels ou aux exigences de Bâle III.
-En conclusion, ce changement est une mise à jour ordinaire des chiffres financiers sans implication méthodologique ou réglementaire. L'analyste peut confirmer cette mise à jour sans nécessiter d'investigation supplémentaire ou d'escalade. Il est recommandé de vérifier la cohérence de ces chiffres avec d'autres sections du rapport pour assurer l'exactitude globale des données financières.</t>
+          <t>La note de bas de page n°3 a subi une modification mineure dans le tableau des actifs grevés et non grevés. Le texte a été mis à jour pour refléter un changement dans le montant des valeurs mobilières, passant de 25,9 milliards de dollars au 31 janvier 2025 à 24,9 milliards de dollars au 30 avril 2025. Cette modification est purement quantitative et ne change pas la nature ou la portée des actifs décrits.
+L'impact de ce changement est principalement cosmétique, car il ne modifie pas la méthodologie ou les critères d'évaluation des actifs non grevés. Il s'agit d'une mise à jour ordinaire des chiffres financiers pour refléter les données les plus récentes. Aucune implication réglementaire ou méthodologique significative n'est associée à cette modification, car elle ne touche pas aux principes sous-jacents de la gestion des risques ou de la conformité aux normes IFRS.
+En conclusion, cette mise à jour est une révision ordinaire des données financières. L'analyste peut confirmer cette mise à jour sans nécessiter d'investigation supplémentaire, car elle ne présente pas de risque ou de changement structurel nécessitant une escalade.</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1228,8 +1224,8 @@
       <c r="I12" s="4" t="inlineStr">
         <is>
           <t>La note de bas de page n-4 a été mise à jour pour refléter les nouvelles valeurs du financement de gros en dollars canadiens et en devises étrangères. Les montants sont passés de 52,3 milliards à 53,0 milliards de dollars canadiens et de 211,1 milliards à 205,8 milliards de dollars américains et autres monnaies.
-Ce changement est principalement une mise à jour des chiffres financiers pour le trimestre en cours. Il reflète les variations dans la composition monétaire du financement de gros, ce qui peut être dû à des fluctuations de change ou à des ajustements dans la stratégie de financement de l'institution. Bien que ces chiffres soient importants pour l'analyse financière, ils ne représentent pas un changement méthodologique ou réglementaire.
-Il s'agit d'une mise à jour ordinaire des données financières. L'analyste devrait confirmer que ces chiffres sont cohérents avec les autres sections du rapport financier et qu'ils reflètent fidèlement la situation financière actuelle de l'institution.</t>
+Ce changement est principalement une mise à jour des chiffres financiers pour le trimestre en cours. Il reflète les variations dans la composition monétaire du financement de gros, ce qui est une pratique courante dans les rapports financiers trimestriels. Bien que cela n'ait pas d'impact direct sur les exigences réglementaires, cela peut influencer l'analyse des tendances financières et la gestion des risques de change.
+Il s'agit d'une mise à jour ordinaire des chiffres financiers. L'analyste devrait confirmer que ces chiffres sont cohérents avec les autres sections du rapport financier et qu'ils reflètent fidèlement les conditions de marché actuelles.</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1250,44 +1246,40 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>TABLEAU 39</t>
+          <t>TABLEAU 36</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>47</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>51</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Note de bas de page</t>
+          <t>Indicateur</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Modification</t>
+          <t>Suppression</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Des dépôts de 29 063 millions de dollars au 31 janvier 2025 ont une date d’échéance fixe, mais ils peuvent toutefois faire l’objet d’une demande de remboursement anticipé (en totalité ou en partie) par le client sans pénalité. Ils sont classés comme étant exigibles à une date fixe en raison de leur date d’échéance contractuelle déclarée.</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>Des dépôts de 28 685 millions de dollars au 30 avril 2025 ont une date d’échéance fixe, mais ils peuvent toutefois faire l’objet d’une demande de remboursement anticipé (en totalité ou en partie) par le client sans pénalité. Ils sont classés comme étant exigibles à une date fixe en raison de leur date d’échéance contractuelle déclarée.</t>
-        </is>
-      </c>
+          <t>Pour le trimestre clos le 31 octobre 2024 – Total des sorties nettes de trésorerie</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr"/>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>La note de bas de page n°3 a été mise à jour pour refléter un changement de montant et de date, passant de 29 063 millions de dollars au 31 janvier 2025 à 28 685 millions de dollars au 30 avril 2025. Cette note est liée aux dépôts ayant une date d’échéance fixe mais pouvant être remboursés anticipativement.
-Ce changement est purement factuel et reflète une mise à jour des données financières pour le trimestre en cours. Il n'affecte pas la méthodologie de calcul des échéances ni les obligations de divulgation réglementaire. Les principes de classification restent inchangés, conformément aux normes IFRS et aux directives du BSIF.
-Il s'agit d'une mise à jour ordinaire des données financières. L'analyste peut confirmer que cette modification est conforme aux pratiques de mise à jour trimestrielle et ne nécessite pas d'investigation supplémentaire.</t>
+          <t>L'indicateur "Pour le trimestre clos le 31 octobre 2024 – Total des sorties nettes de trésorerie" a été retiré du tableau de gestion des risques au T2 2025, alors qu'il était présent au T1 2025.
+Ce retrait semble être une simplification de la présentation des données historiques, probablement pour éviter la redondance avec les nouvelles lignes ajoutées. Cela n'affecte pas directement les exigences réglementaires mais peut influencer la clarté des rapports pour les utilisateurs finaux.
+Il s'agit d'une mise à jour cosmétique. L'analyste devrait vérifier que les informations pertinentes sont toujours disponibles ailleurs dans le rapport.</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1296,9 +1288,21 @@
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr"/>
-      <c r="L13" s="4" t="inlineStr"/>
-      <c r="M13" s="4" t="inlineStr"/>
-      <c r="N13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-19T00:10:18.738993+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1308,17 +1312,17 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>TABLEAU 42</t>
+          <t>TABLEAU 39</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>49</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>53</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1343,9 +1347,9 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>La note de bas de page n°1 a subi une légère modification de formulation, passant de 'Sans échéance' à 'Sans échéance spécifique'. Cette modification concerne le tableau des échéances des passifs et capitaux propres, qui est un élément clé de la gestion des risques de liquidité de la banque.
-Bien que le changement de formulation semble mineur, il pourrait refléter une tentative de clarification de la terminologie utilisée pour décrire les échéances des prêts à vue. Cela pourrait avoir un impact sur la manière dont les informations sont interprétées par les parties prenantes, mais il n'y a pas d'implication réglementaire directe ou de changement méthodologique apparent lié à Bâle III ou aux exigences du BSIF.
-Ce changement est principalement cosmétique et vise à améliorer la clarté du rapport. L'analyste devrait confirmer que cette modification n'entraîne pas de confusion supplémentaire et qu'elle est cohérente avec d'autres sections du rapport.</t>
+          <t>La note de bas de page n°1 a subi une légère modification de formulation, passant de 'Sans échéance' à 'Sans échéance spécifique'. Cette modification concerne le tableau des échéances des passifs et capitaux propres, qui est un élément clé de la gestion des risques de liquidité.
+Cette reformulation n'a pas d'impact significatif sur les exigences réglementaires ou les ratios prudentiels, car elle ne modifie pas la méthodologie de calcul ou la classification des prêts à vue. Elle semble viser à clarifier la terminologie utilisée, potentiellement pour aligner le langage avec d'autres sections du rapport ou avec des normes internes de présentation.
+Il s'agit d'une mise à jour cosmétique. L'analyste peut confirmer que cette modification n'entraîne pas de changement dans les pratiques de divulgation ou de calcul, mais aucune action supplémentaire n'est nécessaire.</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1366,7 +1370,7 @@
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>2026-04-18T19:06:51.386666+00:00</t>
+          <t>2026-04-19T00:10:35.396521+00:00</t>
         </is>
       </c>
     </row>
@@ -1378,17 +1382,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>TABLEAU 42</t>
+          <t>TABLEAU 39</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>49</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>53</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1413,9 +1417,9 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>La note de bas de page n°2 a été modifiée pour inclure le terme 'spécifique' après 'Sans échéance'. Cette modification apparaît dans le même tableau des échéances des passifs et capitaux propres, qui est essentiel pour l'analyse de la liquidité et des engagements de la banque.
-L'ajout du mot 'spécifique' semble être une clarification terminologique sans impact direct sur les calculs ou les ratios prudentiels. Il n'y a pas de changement dans la méthodologie de calcul des échéances ou des dépôts, et cela ne semble pas affecter les exigences de divulgation réglementaire.
-Ce changement est considéré comme cosmétique et vise à améliorer la précision du langage utilisé dans le rapport. L'analyste devrait s'assurer que cette modification est bien comprise par les lecteurs du rapport et qu'elle est appliquée de manière cohérente dans d'autres documents connexes.</t>
+          <t>La note de bas de page n°2 a été reformulée pour inclure le terme 'Sans échéance spécifique' au lieu de 'Sans échéance'. Cette modification apparaît dans le même tableau des échéances des passifs et capitaux propres, et concerne les dépôts à vue et à préavis.
+Cette modification n'affecte pas les obligations réglementaires ou les calculs de ratios, car elle ne change pas la nature des dépôts ou leur classification. Elle semble être une clarification terminologique, probablement pour assurer une cohérence dans la terminologie utilisée à travers le document ou pour répondre à des normes internes de présentation.
+Il s'agit d'une mise à jour cosmétique. L'analyste devrait vérifier que cette modification n'impacte pas d'autres sections du rapport, mais aucune action corrective n'est requise.</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1424,84 +1428,258 @@
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr"/>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M15" s="4" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N15" s="4" t="inlineStr">
-        <is>
-          <t>2026-04-18T19:07:34.344781+00:00</t>
-        </is>
-      </c>
+      <c r="L15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr"/>
+      <c r="N15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>TABLEAU 39</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Note de bas de page</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Des dépôts de 29 063 millions de dollars au 31 janvier 2025 ont une date d’échéance fixe, mais ils peuvent toutefois faire l’objet d’une demande de remboursement anticipé (en totalité ou en partie) par le client sans pénalité. Ils sont classés comme étant exigibles à une date fixe en raison de leur date d’échéance contractuelle déclarée.</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Des dépôts de 28 685 millions de dollars au 30 avril 2025 ont une date d’échéance fixe, mais ils peuvent toutefois faire l’objet d’une demande de remboursement anticipé (en totalité ou en partie) par le client sans pénalité. Ils sont classés comme étant exigibles à une date fixe en raison de leur date d’échéance contractuelle déclarée.</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>La note de bas de page n°3 a été mise à jour pour refléter un changement de montant et de date, passant de 29 063 millions de dollars au 31 janvier 2025 à 28 685 millions de dollars au 30 avril 2025. Cette note est liée aux dépôts ayant une date d’échéance fixe mais pouvant être remboursés anticipativement.
+Ce changement est purement factuel et reflète une mise à jour des données financières pour le trimestre en cours. Il n'affecte pas les méthodologies de calcul ou les exigences réglementaires, car il s'agit simplement d'une actualisation des chiffres pour refléter la situation actuelle.
+Il s'agit d'une mise à jour ordinaire des données financières. L'analyste peut confirmer que les chiffres sont corrects et alignés avec les autres sections du rapport, mais aucune action supplémentaire n'est nécessaire.</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr"/>
+      <c r="N16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>TABLEAU 42</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Note de bas de page</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Les prêts à vue sont inclus dans la colonne Sans échéance.</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Les prêts à vue sont inclus dans la colonne Sans échéance spécifique.</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>La note de bas de page n°1 a subi une légère modification de texte, passant de 'Sans échéance' à 'Sans échéance spécifique'. Cette modification concerne le tableau des échéances des passifs et capitaux propres, qui est un élément clé de la gestion des risques de liquidité de la banque.
+L'impact de ce changement est principalement cosmétique, car il ne modifie pas la méthodologie de classification des prêts à vue. Cependant, l'ajout du terme 'spécifique' pourrait être interprété comme une clarification visant à renforcer la précision du langage utilisé dans les rapports financiers, ce qui est conforme aux bonnes pratiques de divulgation.
+Il s'agit d'une mise à jour ordinaire qui ne nécessite pas d'action immédiate. L'analyste peut confirmer que cette modification n'a pas d'impact sur les calculs ou les ratios prudentiels, mais il n'est pas nécessaire d'escalader ce changement.</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-19T00:10:38.577736+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>TABLEAU 42</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Note de bas de page</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Les dépôts à vue et à préavis sont inclus dans la colonne Sans échéance.</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Les dépôts à vue et à préavis sont inclus dans la colonne Sans échéance spécifique.</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>La note de bas de page n°2 a été modifiée pour inclure le terme 'spécifique' après 'Sans échéance'. Cette note se trouve dans le même tableau des échéances des passifs et capitaux propres, et elle concerne la classification des dépôts à vue et à préavis.
+L'ajout du mot 'spécifique' ne change pas la substance de la note, mais il peut être perçu comme une tentative d'améliorer la clarté et la précision du rapport. Cela peut être particulièrement pertinent dans le contexte de la communication avec les parties prenantes externes, telles que les régulateurs ou les investisseurs, qui exigent une transparence accrue.
+Cette modification est considérée comme cosmétique et ne nécessite pas d'investigation approfondie. L'analyste devrait simplement confirmer que cette clarification n'affecte pas les pratiques de divulgation ou les calculs sous-jacents.</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="inlineStr"/>
+      <c r="N18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
           <t>Réglementation</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>TABLEAU 21</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Tableau</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Suppression</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>TABLEAU 21</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr"/>
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Tableau supprimé du trimestre courant.</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr">
         <is>
           <t>Validé</t>
         </is>
       </c>
-      <c r="M16" s="4" t="inlineStr">
+      <c r="M19" s="4" t="inlineStr">
         <is>
           <t>analyst</t>
         </is>
       </c>
-      <c r="N16" s="4" t="inlineStr">
-        <is>
-          <t>2026-04-18T19:07:26.977810+00:00</t>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-19T00:11:04.168490+00:00</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N16"/>
+  <autoFilter ref="A1:N19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
adding result of T4-BMO
</commit_message>
<xml_diff>
--- a/outputs/resultats/bmo/2025_t2_vs_2025_t1/comparison.xlsx
+++ b/outputs/resultats/bmo/2025_t2_vs_2025_t1/comparison.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changements détectés" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changements détectés'!$A$1:$N$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changements détectés'!$A$1:$M$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -469,11 +469,10 @@
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
     <col width="70" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -524,7 +523,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Nouvelle divulgation ?</t>
+          <t>Nouvelle idée ?</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -538,11 +537,6 @@
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Validé par</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Validé le</t>
         </is>
@@ -602,21 +596,8 @@
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:10:59.190392+00:00</t>
-        </is>
-      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -670,7 +651,6 @@
       <c r="K3" s="3" t="inlineStr"/>
       <c r="L3" s="3" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
-      <c r="N3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -726,21 +706,8 @@
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:10:36.694576+00:00</t>
-        </is>
-      </c>
+      <c r="L4" s="3" t="inlineStr"/>
+      <c r="M4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -798,7 +765,6 @@
       <c r="K5" s="3" t="inlineStr"/>
       <c r="L5" s="3" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
-      <c r="N5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -850,21 +816,8 @@
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr"/>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:10:46.154438+00:00</t>
-        </is>
-      </c>
+      <c r="L6" s="3" t="inlineStr"/>
+      <c r="M6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -918,7 +871,6 @@
       <c r="K7" s="3" t="inlineStr"/>
       <c r="L7" s="3" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
-      <c r="N7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -977,12 +929,7 @@
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N8" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:10:15.112415+00:00</t>
+          <t>2026-06-25T15:31:27.421677+00:00</t>
         </is>
       </c>
     </row>
@@ -1040,21 +987,8 @@
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr"/>
-      <c r="L9" s="3" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M9" s="3" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N9" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:11:18.100025+00:00</t>
-        </is>
-      </c>
+      <c r="L9" s="3" t="inlineStr"/>
+      <c r="M9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1106,21 +1040,8 @@
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr"/>
-      <c r="L10" s="3" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M10" s="3" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N10" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:11:43.591641+00:00</t>
-        </is>
-      </c>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1178,7 +1099,6 @@
       <c r="K11" s="4" t="inlineStr"/>
       <c r="L11" s="4" t="inlineStr"/>
       <c r="M11" s="4" t="inlineStr"/>
-      <c r="N11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1236,7 +1156,6 @@
       <c r="K12" s="4" t="inlineStr"/>
       <c r="L12" s="4" t="inlineStr"/>
       <c r="M12" s="4" t="inlineStr"/>
-      <c r="N12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1288,21 +1207,8 @@
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr"/>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M13" s="4" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:10:18.738993+00:00</t>
-        </is>
-      </c>
+      <c r="L13" s="4" t="inlineStr"/>
+      <c r="M13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1358,21 +1264,8 @@
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr"/>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M14" s="4" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:10:35.396521+00:00</t>
-        </is>
-      </c>
+      <c r="L14" s="4" t="inlineStr"/>
+      <c r="M14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1430,7 +1323,6 @@
       <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="4" t="inlineStr"/>
       <c r="M15" s="4" t="inlineStr"/>
-      <c r="N15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1488,7 +1380,6 @@
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1544,21 +1435,8 @@
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr"/>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M17" s="4" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N17" s="4" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:10:38.577736+00:00</t>
-        </is>
-      </c>
+      <c r="L17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1616,7 +1494,6 @@
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1662,24 +1539,11 @@
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr"/>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M19" s="4" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N19" s="4" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:11:04.168490+00:00</t>
-        </is>
-      </c>
+      <c r="L19" s="4" t="inlineStr"/>
+      <c r="M19" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N19"/>
+  <autoFilter ref="A1:M19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>